<commit_message>
Keep charts byte for byte with their style, colors, shapes and data
Charts were rewritten as openpyxl understands them: the chart style and
colors parts, the Excel 2010 style (mc:AlternateContent), chart extensions
and anything else openpyxl does not read were dropped without a warning.

- The chart XML is exported as stored; the parts it uses (chart style,
  colors, user shapes, embedded workbook) go to data/charts/, pictures to
  data/media/, and are restored with the same relationship ids.
- A chart that refers to anything else is exported as openpyxl reads it,
  with a warning.
- Example 04's first chart has a colors part, the Excel 2010 style and an
  Excel 2016 extension.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019UZs6wsi5TT3GKqgC7bYeY
</commit_message>
<xml_diff>
--- a/examples/04-images-charts.xlsx
+++ b/examples/04-images-charts.xlsx
@@ -141,6 +141,14 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
   <chart>
     <title>
       <tx>
@@ -257,6 +265,13 @@
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
+  <extLst>
+    <ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+      <c16r3:dataDisplayOptions16>
+        <c16r3:dispNaAsBlank val="1"/>
+      </c16r3:dataDisplayOptions16>
+    </ext>
+  </extLst>
 </chartSpace>
 </file>
 
@@ -916,6 +931,46 @@
     <dispBlanksAs val="gap"/>
   </chart>
 </chartSpace>
+</file>
+
+<file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
 </file>
 
 <file path=xl/chartsheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>